<commit_message>
added HH table1 code
added HH table1 code
</commit_message>
<xml_diff>
--- a/__READ ME.xlsx
+++ b/__READ ME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="203" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ECFF182C-239F-A04F-A0D5-6167A03F69D3}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A1B0E5DA-E804-7E44-9E71-F75CA95E4194}"/>
   <bookViews>
-    <workbookView xWindow="45280" yWindow="-5060" windowWidth="38960" windowHeight="20480" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
+    <workbookView xWindow="42300" yWindow="-5960" windowWidth="38960" windowHeight="20480" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="213">
   <si>
     <t>Publication CodeName</t>
   </si>
@@ -667,6 +667,15 @@
   </si>
   <si>
     <t>mostly secondary</t>
+  </si>
+  <si>
+    <t>HerculanoHouzel_etal_2015_Table1.xlsx</t>
+  </si>
+  <si>
+    <t>HerculanoHouzel_etal_2015_Table1.csv</t>
+  </si>
+  <si>
+    <t>https://karger.com/bbe/article-pdf/86/3-4/145/2264694/000437413.pdf</t>
   </si>
 </sst>
 </file>
@@ -1350,6 +1359,10 @@
       <c r="I6" t="s">
         <v>34</v>
       </c>
+      <c r="J6" t="str">
+        <f t="shared" ref="J6:J34" si="0">IF(I6="Y", I6, H6)</f>
+        <v>Y</v>
+      </c>
       <c r="K6" t="s">
         <v>36</v>
       </c>
@@ -1393,7 +1406,7 @@
         <v>24</v>
       </c>
       <c r="J7" t="str">
-        <f t="shared" ref="J7:J34" si="0">IF(I7="Y", I7, H7)</f>
+        <f t="shared" si="0"/>
         <v>41467_2020_14356_MOESM6_ESM.xlsx</v>
       </c>
       <c r="K7" t="s">
@@ -1577,6 +1590,9 @@
       <c r="H11" t="s">
         <v>208</v>
       </c>
+      <c r="I11" t="s">
+        <v>34</v>
+      </c>
       <c r="J11" t="s">
         <v>207</v>
       </c>
@@ -1688,16 +1704,26 @@
       <c r="G14" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H14" s="5"/>
-      <c r="J14">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="H14" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" t="s">
+        <v>211</v>
       </c>
       <c r="K14" t="s">
         <v>36</v>
       </c>
       <c r="L14" t="s">
         <v>26</v>
+      </c>
+      <c r="M14" t="s">
+        <v>37</v>
+      </c>
+      <c r="N14" s="3" t="s">
+        <v>212</v>
       </c>
       <c r="O14" t="s">
         <v>61</v>
@@ -1735,6 +1761,12 @@
       <c r="L15" t="s">
         <v>26</v>
       </c>
+      <c r="M15" t="s">
+        <v>37</v>
+      </c>
+      <c r="N15" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="O15" t="s">
         <v>61</v>
       </c>
@@ -1771,6 +1803,12 @@
       <c r="L16" t="s">
         <v>26</v>
       </c>
+      <c r="M16" t="s">
+        <v>37</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="O16" t="s">
         <v>61</v>
       </c>
@@ -1807,6 +1845,12 @@
       <c r="L17" t="s">
         <v>26</v>
       </c>
+      <c r="M17" t="s">
+        <v>37</v>
+      </c>
+      <c r="N17" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="O17" t="s">
         <v>61</v>
       </c>
@@ -1843,6 +1887,12 @@
       <c r="L18" t="s">
         <v>26</v>
       </c>
+      <c r="M18" t="s">
+        <v>37</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>212</v>
+      </c>
       <c r="O18" t="s">
         <v>61</v>
       </c>
@@ -1878,6 +1928,12 @@
       </c>
       <c r="L19" t="s">
         <v>26</v>
+      </c>
+      <c r="M19" t="s">
+        <v>37</v>
+      </c>
+      <c r="N19" s="3" t="s">
+        <v>212</v>
       </c>
       <c r="O19" t="s">
         <v>61</v>
@@ -2585,12 +2641,23 @@
     <hyperlink ref="N29" r:id="rId34" xr:uid="{C4869E3C-B5B1-6647-A144-091B1A64A38B}"/>
     <hyperlink ref="N30" r:id="rId35" xr:uid="{808C07EB-0E2A-B640-A28C-8E310E5A987B}"/>
     <hyperlink ref="A31" r:id="rId36" xr:uid="{DE23E549-C543-F745-A3C2-B0DDB1E2B18A}"/>
+    <hyperlink ref="N14" r:id="rId37" xr:uid="{9534F0D1-7C63-EC4F-921C-5D21474866A4}"/>
+    <hyperlink ref="N15:N19" r:id="rId38" display="https://karger.com/bbe/article-pdf/86/3-4/145/2264694/000437413.pdf" xr:uid="{0070BD27-D760-3846-9F0D-91BB5EDD333F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009B0162F312A93D41AE706303C1572F17" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="acb3cbe4b9dee1876b3bbe7116f679b3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8e1efd23-f4ba-42d2-85fd-6a510437bae6" xmlns:ns3="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ca927c27970307cd175704f09b582c5c" ns2:_="" ns3:_="">
     <xsd:import namespace="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
@@ -2827,15 +2894,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2848,6 +2906,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2F6D714A-5497-420A-9146-5640EA73F0F4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2866,27 +2932,19 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
   <ds:schemaRefs>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
code to extract all HH data added
</commit_message>
<xml_diff>
--- a/__READ ME.xlsx
+++ b/__READ ME.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="287" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B7CCB523-DD9C-2142-9C4D-294B5C6C4BAA}"/>
+  <xr:revisionPtr revIDLastSave="291" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0779C6BC-9F46-FE46-B9B1-D42CCBE321FE}"/>
   <bookViews>
-    <workbookView xWindow="1960" yWindow="760" windowWidth="30660" windowHeight="15420" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
+    <workbookView xWindow="280" yWindow="760" windowWidth="33820" windowHeight="19080" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="231">
   <si>
     <t>Publication CodeName</t>
   </si>
@@ -724,9 +724,6 @@
   </si>
   <si>
     <t>docx online</t>
-  </si>
-  <si>
-    <t>units</t>
   </si>
   <si>
     <t>JardimMesseder_etal_2017_Table1.csv</t>
@@ -791,12 +788,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -812,7 +815,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -827,7 +830,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1505,92 +1513,92 @@
         <v>54</v>
       </c>
     </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="13" t="s">
         <v>144</v>
       </c>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="E8" s="7" t="s">
+      <c r="E8" s="13" t="s">
         <v>146</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="12" t="s">
         <v>218</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="L8" t="s">
+      <c r="L8" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M8" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="N8" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="O8" t="s">
+      <c r="O8" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="P8" t="s">
+      <c r="P8" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="S8" t="s">
+      <c r="S8" s="12" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="13" t="s">
         <v>147</v>
       </c>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="13"/>
+      <c r="D9" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" t="s">
+      <c r="E9" s="13"/>
+      <c r="F9" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="5" t="s">
+      <c r="G9" s="14"/>
+      <c r="H9" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="12" t="s">
         <v>217</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="12" t="s">
         <v>219</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O9" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="S9" t="s">
+      <c r="S9" s="12" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1757,319 +1765,319 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+    <row r="14" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7" t="s">
+      <c r="C14" s="13"/>
+      <c r="D14" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" t="s">
+      <c r="E14" s="13"/>
+      <c r="F14" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G14" s="7" t="s">
+      <c r="G14" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="I14" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="12" t="s">
         <v>205</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L14" t="s">
+      <c r="L14" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M14" t="s">
+      <c r="M14" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N14" s="3" t="s">
+      <c r="N14" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="O14" t="s">
+      <c r="O14" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S14" t="s">
+      <c r="S14" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+    <row r="15" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B15" s="7" t="s">
+      <c r="B15" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7" t="s">
+      <c r="C15" s="13"/>
+      <c r="D15" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" t="s">
+      <c r="E15" s="13"/>
+      <c r="F15" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G15" s="7" t="s">
+      <c r="G15" s="13" t="s">
         <v>159</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="15" t="s">
         <v>207</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="I15" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M15" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="N15" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="O15" t="s">
+      <c r="O15" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S15" t="s">
+      <c r="S15" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+    <row r="16" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B16" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7" t="s">
+      <c r="C16" s="13"/>
+      <c r="D16" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" t="s">
+      <c r="E16" s="13"/>
+      <c r="F16" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="G16" s="13" t="s">
         <v>160</v>
       </c>
-      <c r="H16" s="12" t="s">
+      <c r="H16" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="I16" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L16" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M16" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="N16" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="O16" t="s">
+      <c r="O16" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+    <row r="17" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B17" s="7" t="s">
+      <c r="B17" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7" t="s">
+      <c r="C17" s="13"/>
+      <c r="D17" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" t="s">
+      <c r="E17" s="13"/>
+      <c r="F17" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G17" s="8" t="s">
+      <c r="G17" s="17" t="s">
         <v>161</v>
       </c>
-      <c r="H17" s="5" t="s">
+      <c r="H17" s="15" t="s">
         <v>209</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="12" t="s">
         <v>213</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L17" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M17" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="N17" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="O17" t="s">
+      <c r="O17" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S17" t="s">
+      <c r="S17" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
+    <row r="18" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7" t="s">
+      <c r="C18" s="13"/>
+      <c r="D18" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" t="s">
+      <c r="E18" s="13"/>
+      <c r="F18" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G18" s="8" t="s">
+      <c r="G18" s="17" t="s">
         <v>162</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="15" t="s">
         <v>210</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="I18" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="12" t="s">
         <v>214</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L18" t="s">
+      <c r="L18" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M18" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="N18" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="O18" t="s">
+      <c r="O18" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S18" t="s">
+      <c r="S18" s="12" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="7" t="s">
+      <c r="B19" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7" t="s">
+      <c r="C19" s="13"/>
+      <c r="D19" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="E19" s="7"/>
-      <c r="F19" t="s">
+      <c r="E19" s="13"/>
+      <c r="F19" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="G19" s="14" t="s">
         <v>164</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="15" t="s">
         <v>220</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="I19" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L19" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M19" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O19" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="S19" t="s">
+      <c r="S19" s="12" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
+    <row r="20" spans="1:19" s="12" customFormat="1" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="7" t="s">
+      <c r="B20" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7" t="s">
+      <c r="C20" s="13"/>
+      <c r="D20" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="E20" s="7"/>
-      <c r="F20" t="s">
+      <c r="E20" s="13"/>
+      <c r="F20" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="G20" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="H20" s="5" t="s">
+      <c r="H20" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="I20" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="12" t="s">
         <v>222</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L20" t="s">
+      <c r="L20" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M20" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="O20" t="s">
+      <c r="O20" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="S20" t="s">
+      <c r="S20" s="12" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2217,132 +2225,132 @@
         <v>85</v>
       </c>
     </row>
-    <row r="25" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
+    <row r="25" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="B25" s="7" t="s">
+      <c r="B25" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7" t="s">
+      <c r="C25" s="13"/>
+      <c r="D25" s="13" t="s">
         <v>133</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" t="s">
+      <c r="E25" s="13"/>
+      <c r="F25" s="12" t="s">
         <v>197</v>
       </c>
-      <c r="G25" s="3"/>
-      <c r="H25" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="I25" s="7" t="s">
+      <c r="G25" s="14"/>
+      <c r="H25" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="I25" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J25" t="s">
-        <v>230</v>
-      </c>
-      <c r="K25" t="s">
+      <c r="J25" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="K25" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="L25" t="s">
+      <c r="L25" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M25" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="O25" t="s">
+      <c r="O25" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="S25" t="s">
+      <c r="S25" s="12" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="26" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
+    <row r="26" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7" t="s">
+      <c r="C26" s="13"/>
+      <c r="D26" s="13" t="s">
         <v>145</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" t="s">
-        <v>229</v>
-      </c>
-      <c r="G26" s="3" t="s">
+      <c r="E26" s="13"/>
+      <c r="F26" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="G26" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="H26" s="5"/>
-      <c r="I26" s="7" t="s">
+      <c r="H26" s="15"/>
+      <c r="I26" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="12" t="s">
         <v>226</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="L26" t="s">
+      <c r="L26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M26" t="s">
+      <c r="M26" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N26" s="3" t="s">
+      <c r="N26" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="O26" t="s">
+      <c r="O26" s="12" t="s">
         <v>168</v>
       </c>
-      <c r="S26" t="s">
+      <c r="S26" s="12" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="27" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
+    <row r="27" spans="1:19" s="12" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="B27" s="7" t="s">
+      <c r="B27" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7" t="s">
+      <c r="C27" s="13"/>
+      <c r="D27" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" t="s">
-        <v>229</v>
-      </c>
-      <c r="G27" s="3" t="s">
+      <c r="E27" s="13"/>
+      <c r="F27" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="G27" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="H27" s="5"/>
-      <c r="I27" s="7" t="s">
+      <c r="H27" s="15"/>
+      <c r="I27" s="13" t="s">
         <v>34</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="12" t="s">
         <v>227</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K27" s="12" t="s">
         <v>228</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L27" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="M27" t="s">
+      <c r="M27" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="N27" s="3" t="s">
+      <c r="N27" s="14" t="s">
         <v>225</v>
       </c>
-      <c r="O27" t="s">
+      <c r="O27" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="S27" t="s">
+      <c r="S27" s="12" t="s">
         <v>178</v>
       </c>
     </row>

</xml_diff>

<commit_message>
cell composition data renaming
</commit_message>
<xml_diff>
--- a/__READ ME.xlsx
+++ b/__READ ME.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11116"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://alleninstitute.sharepoint.com/sites/MammalianM1/Shared Documents/General/Species/Evo M1 Trait Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="291" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0779C6BC-9F46-FE46-B9B1-D42CCBE321FE}"/>
+  <xr:revisionPtr revIDLastSave="295" documentId="13_ncr:1_{A611BB1F-8283-7640-98A2-533433C96266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8621A9CB-C081-5C4A-B469-5BAD279D947B}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="760" windowWidth="33820" windowHeight="19080" xr2:uid="{D451F2D8-9E4F-7644-8584-5A4B2BCAED4A}"/>
   </bookViews>
@@ -1156,14 +1156,14 @@
   <cols>
     <col min="1" max="1" width="24.1640625" customWidth="1"/>
     <col min="2" max="2" width="31.6640625" customWidth="1"/>
-    <col min="3" max="3" width="22.33203125" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
     <col min="4" max="4" width="20.83203125" customWidth="1"/>
     <col min="5" max="5" width="23.1640625" customWidth="1"/>
     <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="5.33203125" customWidth="1"/>
-    <col min="10" max="10" width="31" customWidth="1"/>
+    <col min="10" max="10" width="35.33203125" customWidth="1"/>
     <col min="11" max="11" width="13.83203125" customWidth="1"/>
     <col min="12" max="12" width="12.6640625" customWidth="1"/>
     <col min="13" max="13" width="22.1640625" customWidth="1"/>
@@ -2978,15 +2978,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764" xsi:nil="true"/>
@@ -2995,6 +2986,15 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3017,26 +3017,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{025C630B-64D2-4AAA-9CA6-B49D96BBCC82}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B6DEDC7-93D0-4B5E-BED5-006DF8C890FC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="3bad6c6a-329d-45e9-b8b0-1ebecc8a8764"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="8e1efd23-f4ba-42d2-85fd-6a510437bae6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>